<commit_message>
Version 1.1.0: HRDU System with the Leave cards module
- Leave card per employee under the CSC Omnibus Rules on Leave: monthly
  1.25 VL/SL credits less 1/30 per day without pay, tardiness/undertime
  via the CSC conversion table, SL charged to VL when SL runs out, SPL cap,
  monetization (0.0481927), forced leave deducted at year end, terminal
  leave estimate.
- Leave applications on CS Form No. 6 (Revised 2020), printed on long bond
  paper, with signatory drop-downs; an approved leave posts to the card.
- Employee sign-in (role Employee) that sees only its own leave card.
- Tests: dev/test-leave.js (CSC tables and rules), browser flow for leave.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LdEkDbLfqACC1g6rNmky7Q
</commit_message>
<xml_diff>
--- a/Register/HRDU Training Evaluation Register.xlsx
+++ b/Register/HRDU Training Evaluation Register.xlsx
@@ -10,9 +10,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trainings" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Responses" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource Person Ratings" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Users" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Trail" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leave Ledger" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leave Applications" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signatories" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Users" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Trail" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -530,6 +534,48 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>HRDU Training Evaluation Register (HRDU System: Training Evaluation Tool, Level 1, and Leave cards)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Version 1.1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Upload to Google Drive, open, File &gt; Save as Google Sheets, then follow the README (Extensions &gt; Apps Script).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Do not type in the tabs by hand. The app writes to them.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -776,76 +822,118 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Username</t>
+          <t>Employee No.</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Full Name</t>
+          <t>Last Name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Middle Name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Position</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Password</t>
+          <t>Office / Unit</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Must Change Password</t>
+          <t>Status of Appointment</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Last Sign-in</t>
+          <t>Date of Original Appointment</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Leave Card Start</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Monthly Salary</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Highest Monthly Salary</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Employment Status</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Separation Date</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Created At</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Updated At</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Updated By</t>
         </is>
       </c>
     </row>
@@ -855,6 +943,360 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:X1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Entry No.</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Employee No.</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Leave Type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Date From</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Date To</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Times Late</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Minutes</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>VL W/P</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>VL W/O P</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>SL W/P</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>SL W/O P</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>VL Added</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>SL Added</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Action Taken</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Application No.</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Record Status</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Void Reason</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Encoded At</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Encoded By</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AC1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="17" customWidth="1" min="22" max="22"/>
+    <col width="26" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Application No.</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Employee No.</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Date of Filing</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Leave Type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Others Specify</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Details Specify</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Days Applied</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Date From</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Date To</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Inclusive Dates</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Commutation</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Certified As Of</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Certified By</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Recommended By</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Disapproval Reason (7.B)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Approved By</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Days With Pay</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Days Without Pay</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Others Approved</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Disapproved Due To (7.D)</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Decided At</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Entry No.</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Filed By</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Created At</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Updated At</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Updated By</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -874,32 +1316,32 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Signs For</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>By</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Details</t>
+          <t>Updated At</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Updated By</t>
         </is>
       </c>
     </row>
@@ -908,40 +1350,142 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>HRDU Training Evaluation Register (Training Evaluation Tool, Level 1)</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Username</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Full Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Password</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Must Change Password</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Last Sign-in</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Created At</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Updated At</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Employee No.</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Version 1.0.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Upload to Google Drive, open, File &gt; Save as Google Sheets, then follow the README (Extensions &gt; Apps Script).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Do not type in the tabs by hand. The app writes to them.</t>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>By</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Device</t>
         </is>
       </c>
     </row>

</xml_diff>